<commit_message>
Add WBS link to presentation
</commit_message>
<xml_diff>
--- a/docs/LLM_Wiki_WBS_Gantt.xlsx
+++ b/docs/LLM_Wiki_WBS_Gantt.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS &amp; Gantt" sheetId="1" r:id="R6ffe10ab55874d91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Reb5fe54f23f64c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WBS &amp; Gantt" sheetId="1" r:id="R1cab83c97c1c41f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R585d6725f3574ac7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -715,7 +715,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6122a6e323a34d1f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd92701633fd649ed"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1112,9 +1112,7 @@
       <x:c r="B5" s="29" t="str">
         <x:v>기획 및 설계</x:v>
       </x:c>
-      <x:c r="C5" s="28" t="str">
-        <x:v>-</x:v>
-      </x:c>
+      <x:c r="C5" s="28"/>
       <x:c r="D5" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
@@ -1170,9 +1168,7 @@
       <x:c r="B6" s="15" t="str">
         <x:v>프로젝트 기획</x:v>
       </x:c>
-      <x:c r="C6" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C6" s="14"/>
       <x:c r="D6" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1236,9 +1232,7 @@
       <x:c r="B7" s="15" t="str">
         <x:v>비전 및 요구사항 정의</x:v>
       </x:c>
-      <x:c r="C7" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C7" s="14"/>
       <x:c r="D7" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1302,9 +1296,7 @@
       <x:c r="B8" s="15" t="str">
         <x:v>주요 기능 및 보안 요구사항 정리</x:v>
       </x:c>
-      <x:c r="C8" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C8" s="14"/>
       <x:c r="D8" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1368,9 +1360,7 @@
       <x:c r="B9" s="15" t="str">
         <x:v>아키텍처 의사결정 정리</x:v>
       </x:c>
-      <x:c r="C9" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C9" s="14"/>
       <x:c r="D9" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1434,9 +1424,7 @@
       <x:c r="B10" s="15" t="str">
         <x:v>로컬 우선 구조 ADR 작성</x:v>
       </x:c>
-      <x:c r="C10" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C10" s="14"/>
       <x:c r="D10" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1500,9 +1488,7 @@
       <x:c r="B11" s="15" t="str">
         <x:v>BYOK / 마크다운 / 플러터 ADR 작성</x:v>
       </x:c>
-      <x:c r="C11" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C11" s="14"/>
       <x:c r="D11" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1566,9 +1552,7 @@
       <x:c r="B12" s="15" t="str">
         <x:v>발표 및 프로젝트 문서화</x:v>
       </x:c>
-      <x:c r="C12" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C12" s="14"/>
       <x:c r="D12" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1632,9 +1616,7 @@
       <x:c r="B13" s="15" t="str">
         <x:v>PRD / ADR / README 정리</x:v>
       </x:c>
-      <x:c r="C13" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C13" s="14"/>
       <x:c r="D13" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1698,9 +1680,7 @@
       <x:c r="B14" s="45" t="str">
         <x:v>1차 산출물 점검</x:v>
       </x:c>
-      <x:c r="C14" s="44" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C14" s="44"/>
       <x:c r="D14" s="44" t="str">
         <x:v>Milestone</x:v>
       </x:c>
@@ -1766,9 +1746,7 @@
       <x:c r="B15" s="29" t="str">
         <x:v>개발 환경 구축</x:v>
       </x:c>
-      <x:c r="C15" s="28" t="str">
-        <x:v>-</x:v>
-      </x:c>
+      <x:c r="C15" s="28"/>
       <x:c r="D15" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
@@ -1824,9 +1802,7 @@
       <x:c r="B16" s="15" t="str">
         <x:v>프로젝트 초기화</x:v>
       </x:c>
-      <x:c r="C16" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C16" s="14"/>
       <x:c r="D16" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1890,9 +1866,7 @@
       <x:c r="B17" s="15" t="str">
         <x:v>Flutter 프로젝트 생성</x:v>
       </x:c>
-      <x:c r="C17" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C17" s="14"/>
       <x:c r="D17" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -1956,9 +1930,7 @@
       <x:c r="B18" s="15" t="str">
         <x:v>GitHub Repository 및 Pages 설정</x:v>
       </x:c>
-      <x:c r="C18" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C18" s="14"/>
       <x:c r="D18" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -2022,9 +1994,7 @@
       <x:c r="B19" s="15" t="str">
         <x:v>기본 앱 UI 구성</x:v>
       </x:c>
-      <x:c r="C19" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C19" s="14"/>
       <x:c r="D19" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -2088,9 +2058,7 @@
       <x:c r="B20" s="15" t="str">
         <x:v>라이브러리 / 캡처 / 내보내기 / 보안 화면</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C20" s="14"/>
       <x:c r="D20" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -2154,9 +2122,7 @@
       <x:c r="B21" s="15" t="str">
         <x:v>발표용 GitHub Pages 구성</x:v>
       </x:c>
-      <x:c r="C21" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C21" s="14"/>
       <x:c r="D21" s="33" t="str">
         <x:v>Completed</x:v>
       </x:c>
@@ -2220,9 +2186,7 @@
       <x:c r="B22" s="45" t="str">
         <x:v>개발 환경 점검</x:v>
       </x:c>
-      <x:c r="C22" s="44" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C22" s="44"/>
       <x:c r="D22" s="44" t="str">
         <x:v>Milestone</x:v>
       </x:c>
@@ -2288,9 +2252,7 @@
       <x:c r="B23" s="29" t="str">
         <x:v>도메인 및 데이터 레이어</x:v>
       </x:c>
-      <x:c r="C23" s="28" t="str">
-        <x:v>-</x:v>
-      </x:c>
+      <x:c r="C23" s="28"/>
       <x:c r="D23" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
@@ -2346,9 +2308,7 @@
       <x:c r="B24" s="15" t="str">
         <x:v>도메인 모델 정리</x:v>
       </x:c>
-      <x:c r="C24" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C24" s="14"/>
       <x:c r="D24" s="49" t="str">
         <x:v>In progress</x:v>
       </x:c>
@@ -2412,9 +2372,7 @@
       <x:c r="B25" s="15" t="str">
         <x:v>Conversation / Message / Project 모델</x:v>
       </x:c>
-      <x:c r="C25" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C25" s="14"/>
       <x:c r="D25" s="49" t="str">
         <x:v>In progress</x:v>
       </x:c>
@@ -2478,9 +2436,7 @@
       <x:c r="B26" s="15" t="str">
         <x:v>Repository 인터페이스 분리</x:v>
       </x:c>
-      <x:c r="C26" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C26" s="14"/>
       <x:c r="D26" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -2544,9 +2500,7 @@
       <x:c r="B27" s="15" t="str">
         <x:v>로컬 데이터 저장소 구현</x:v>
       </x:c>
-      <x:c r="C27" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C27" s="14"/>
       <x:c r="D27" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -2610,9 +2564,7 @@
       <x:c r="B28" s="15" t="str">
         <x:v>SQLite 스키마 및 초기화</x:v>
       </x:c>
-      <x:c r="C28" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C28" s="14"/>
       <x:c r="D28" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -2676,9 +2628,7 @@
       <x:c r="B29" s="15" t="str">
         <x:v>대화/메시지/태그 Repository 구현</x:v>
       </x:c>
-      <x:c r="C29" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C29" s="14"/>
       <x:c r="D29" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -2742,9 +2692,7 @@
       <x:c r="B30" s="45" t="str">
         <x:v>중간 점검: 데이터 저장 구조 확인</x:v>
       </x:c>
-      <x:c r="C30" s="44" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C30" s="44"/>
       <x:c r="D30" s="44" t="str">
         <x:v>Milestone</x:v>
       </x:c>
@@ -2810,9 +2758,7 @@
       <x:c r="B31" s="29" t="str">
         <x:v>AI 채팅 및 지식화 기능</x:v>
       </x:c>
-      <x:c r="C31" s="28" t="str">
-        <x:v>-</x:v>
-      </x:c>
+      <x:c r="C31" s="28"/>
       <x:c r="D31" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
@@ -2868,9 +2814,7 @@
       <x:c r="B32" s="15" t="str">
         <x:v>OpenAI API 연동</x:v>
       </x:c>
-      <x:c r="C32" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C32" s="14"/>
       <x:c r="D32" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -2934,9 +2878,7 @@
       <x:c r="B33" s="15" t="str">
         <x:v>BYOK 기반 API 키 입력/검증</x:v>
       </x:c>
-      <x:c r="C33" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C33" s="14"/>
       <x:c r="D33" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3000,9 +2942,7 @@
       <x:c r="B34" s="15" t="str">
         <x:v>채팅 요청/응답 Provider 구현</x:v>
       </x:c>
-      <x:c r="C34" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C34" s="14"/>
       <x:c r="D34" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3066,9 +3006,7 @@
       <x:c r="B35" s="15" t="str">
         <x:v>지식화 자동 처리</x:v>
       </x:c>
-      <x:c r="C35" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C35" s="14"/>
       <x:c r="D35" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3132,9 +3070,7 @@
       <x:c r="B36" s="15" t="str">
         <x:v>태그 생성 및 코드 스니펫 추출</x:v>
       </x:c>
-      <x:c r="C36" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C36" s="14"/>
       <x:c r="D36" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3198,9 +3134,7 @@
       <x:c r="B37" s="15" t="str">
         <x:v>요약 생성 및 프로젝트 분류 보완</x:v>
       </x:c>
-      <x:c r="C37" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C37" s="14"/>
       <x:c r="D37" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3264,9 +3198,7 @@
       <x:c r="B38" s="29" t="str">
         <x:v>검색, 내보내기, 보안</x:v>
       </x:c>
-      <x:c r="C38" s="28" t="str">
-        <x:v>-</x:v>
-      </x:c>
+      <x:c r="C38" s="28"/>
       <x:c r="D38" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
@@ -3322,9 +3254,7 @@
       <x:c r="B39" s="15" t="str">
         <x:v>검색 기능 구현</x:v>
       </x:c>
-      <x:c r="C39" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C39" s="14"/>
       <x:c r="D39" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3388,9 +3318,7 @@
       <x:c r="B40" s="15" t="str">
         <x:v>제목/본문/태그 검색</x:v>
       </x:c>
-      <x:c r="C40" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C40" s="14"/>
       <x:c r="D40" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3454,9 +3382,7 @@
       <x:c r="B41" s="15" t="str">
         <x:v>검색 필터 및 결과 정렬</x:v>
       </x:c>
-      <x:c r="C41" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C41" s="14"/>
       <x:c r="D41" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3520,9 +3446,7 @@
       <x:c r="B42" s="15" t="str">
         <x:v>마크다운 내보내기</x:v>
       </x:c>
-      <x:c r="C42" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C42" s="14"/>
       <x:c r="D42" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3586,9 +3510,7 @@
       <x:c r="B43" s="15" t="str">
         <x:v>Export 포맷 및 Frontmatter 정리</x:v>
       </x:c>
-      <x:c r="C43" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C43" s="14"/>
       <x:c r="D43" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3652,9 +3574,7 @@
       <x:c r="B44" s="15" t="str">
         <x:v>파일 저장 / 공유 기능 연결</x:v>
       </x:c>
-      <x:c r="C44" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C44" s="14"/>
       <x:c r="D44" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3718,9 +3638,7 @@
       <x:c r="B45" s="15" t="str">
         <x:v>보안 기능 구현</x:v>
       </x:c>
-      <x:c r="C45" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C45" s="14"/>
       <x:c r="D45" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3784,9 +3702,7 @@
       <x:c r="B46" s="15" t="str">
         <x:v>Secure Storage / 민감정보 마스킹</x:v>
       </x:c>
-      <x:c r="C46" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C46" s="14"/>
       <x:c r="D46" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3850,9 +3766,7 @@
       <x:c r="B47" s="15" t="str">
         <x:v>앱 잠금 / DB 암호화 검토</x:v>
       </x:c>
-      <x:c r="C47" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C47" s="14"/>
       <x:c r="D47" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -3916,9 +3830,7 @@
       <x:c r="B48" s="29" t="str">
         <x:v>테스트 및 발표 준비</x:v>
       </x:c>
-      <x:c r="C48" s="28" t="str">
-        <x:v>-</x:v>
-      </x:c>
+      <x:c r="C48" s="28"/>
       <x:c r="D48" s="28" t="str">
         <x:v>-</x:v>
       </x:c>
@@ -3974,9 +3886,7 @@
       <x:c r="B49" s="15" t="str">
         <x:v>기능 테스트</x:v>
       </x:c>
-      <x:c r="C49" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C49" s="14"/>
       <x:c r="D49" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -4040,9 +3950,7 @@
       <x:c r="B50" s="15" t="str">
         <x:v>위젯 테스트 / 정적 분석</x:v>
       </x:c>
-      <x:c r="C50" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C50" s="14"/>
       <x:c r="D50" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -4106,9 +4014,7 @@
       <x:c r="B51" s="15" t="str">
         <x:v>모바일/웹 화면 점검</x:v>
       </x:c>
-      <x:c r="C51" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C51" s="14"/>
       <x:c r="D51" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -4172,9 +4078,7 @@
       <x:c r="B52" s="15" t="str">
         <x:v>최종 발표 준비</x:v>
       </x:c>
-      <x:c r="C52" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C52" s="14"/>
       <x:c r="D52" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -4238,9 +4142,7 @@
       <x:c r="B53" s="15" t="str">
         <x:v>GitHub Pages 발표자료 최종 수정</x:v>
       </x:c>
-      <x:c r="C53" s="14" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C53" s="14"/>
       <x:c r="D53" s="50" t="str">
         <x:v>Not Started</x:v>
       </x:c>
@@ -4304,9 +4206,7 @@
       <x:c r="B54" s="45" t="str">
         <x:v>최종 발표 및 제출</x:v>
       </x:c>
-      <x:c r="C54" s="44" t="str">
-        <x:v>윤서호</x:v>
-      </x:c>
+      <x:c r="C54" s="44"/>
       <x:c r="D54" s="44" t="str">
         <x:v>Milestone</x:v>
       </x:c>
@@ -4541,6 +4441,6 @@
     <x:mergeCell ref="A1:D1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfd3a988bbed4961"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09a877d9f4fd4480"/>
 </x:worksheet>
 </file>
</xml_diff>